<commit_message>
Regenerate all example config workbooks with updated schema targets and expr source_ref
- Changed all example configs from sqlite to postgres targets with dedicated schemas (uuid_keys, data_types, broken, stock, showcase)
- Updated kitchen_sink example: order_month now uses expr:{order_date} instead of col:C to demonstrate computed column references
- Regenerated all 17 example config workbooks via make_examples.py
- Updated check-parser skill docs: added test-examples.sh usage, expanded expected
</commit_message>
<xml_diff>
--- a/examples/03_uuid_keys/orders_config.xlsx
+++ b/examples/03_uuid_keys/orders_config.xlsx
@@ -779,7 +779,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>sqlite</t>
+          <t>postgres</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>orders.db</t>
+          <t>excel_parser</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -809,6 +809,11 @@
       <c r="A4" t="inlineStr">
         <is>
           <t>db_schema</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>uuid_keys</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>